<commit_message>
fix: service fee text nowrap
</commit_message>
<xml_diff>
--- a/scratch/test_output_v3.xlsx
+++ b/scratch/test_output_v3.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="874" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="928" uniqueCount="117">
   <si>
     <t>※ 분석 제외 사례수: 0건</t>
   </si>
@@ -572,10 +572,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -4568,272 +4568,356 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A2:H25"/>
+  <dimension ref="A2:J25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="7" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:10">
       <c r="A2" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:10">
       <c r="A3" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="D3" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="E3" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="F3" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="G3" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="H3" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="I3" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="J3" s="9" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:10">
       <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="10">
+      <c r="D4" s="11">
         <v>0.04166666666666666</v>
       </c>
-      <c r="C4" s="10">
+      <c r="E4" s="11">
         <v>0.04166666666666666</v>
       </c>
-      <c r="D4" s="10">
+      <c r="F4" s="11">
         <v>0.04166666666666666</v>
       </c>
-      <c r="G4" s="11" t="s">
+      <c r="I4" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="H4" s="11"/>
-    </row>
-    <row r="5" spans="1:8">
+      <c r="J4" s="10"/>
+    </row>
+    <row r="5" spans="1:10">
       <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="10">
+      <c r="D5" s="11">
         <v>0.04166666666666666</v>
       </c>
-      <c r="C5" s="10">
+      <c r="E5" s="11">
         <v>0.04166666666666666</v>
       </c>
-      <c r="D5" s="10">
+      <c r="F5" s="11">
         <v>0.04166666666666666</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="I5" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="H5" s="11"/>
-    </row>
-    <row r="6" spans="1:8">
+      <c r="J5" s="10"/>
+    </row>
+    <row r="6" spans="1:10">
       <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="10">
+      <c r="D6" s="11">
         <v>0.04166666666666666</v>
       </c>
-      <c r="C6" s="10">
+      <c r="E6" s="11">
         <v>0.04166666666666666</v>
       </c>
-      <c r="D6" s="10">
+      <c r="F6" s="11">
         <v>0.04166666666666666</v>
       </c>
-      <c r="G6" s="11" t="s">
+      <c r="I6" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="H6" s="11"/>
-    </row>
-    <row r="7" spans="1:8">
+      <c r="J6" s="10"/>
+    </row>
+    <row r="7" spans="1:10">
       <c r="A7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="10">
+      <c r="D7" s="11">
         <v>0.04166666666666666</v>
       </c>
-      <c r="C7" s="10">
+      <c r="E7" s="11">
         <v>0.04166666666666666</v>
       </c>
-      <c r="D7" s="10">
+      <c r="F7" s="11">
         <v>0.04166666666666666</v>
       </c>
-      <c r="G7" s="11" t="s">
+      <c r="I7" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="H7" s="11"/>
-    </row>
-    <row r="8" spans="1:8">
+      <c r="J7" s="10"/>
+    </row>
+    <row r="8" spans="1:10">
       <c r="A8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="10">
+      <c r="D8" s="11">
         <v>0.08333333333333333</v>
       </c>
-      <c r="C8" s="10">
+      <c r="E8" s="11">
         <v>0.08333333333333333</v>
       </c>
-      <c r="D8" s="10">
+      <c r="F8" s="11">
         <v>0.08333333333333333</v>
       </c>
-      <c r="G8" s="11" t="s">
+      <c r="I8" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="H8" s="11"/>
-    </row>
-    <row r="9" spans="1:8">
+      <c r="J8" s="10"/>
+    </row>
+    <row r="9" spans="1:10">
       <c r="A9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="10">
+      <c r="D9" s="11">
         <v>0.08333333333333333</v>
       </c>
-      <c r="C9" s="10">
+      <c r="E9" s="11">
         <v>0.08333333333333333</v>
       </c>
-      <c r="D9" s="10">
+      <c r="F9" s="11">
         <v>0.08333333333333333</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="I9" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="H9" s="11"/>
-    </row>
-    <row r="10" spans="1:8">
+      <c r="J9" s="10"/>
+    </row>
+    <row r="10" spans="1:10">
       <c r="A10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="10">
+      <c r="D10" s="11">
         <v>0.08333333333333333</v>
       </c>
-      <c r="C10" s="10">
+      <c r="E10" s="11">
         <v>0.08333333333333333</v>
       </c>
-      <c r="D10" s="10">
+      <c r="F10" s="11">
         <v>0.08333333333333333</v>
       </c>
-      <c r="G10" s="11" t="s">
+      <c r="I10" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="H10" s="11"/>
-    </row>
-    <row r="11" spans="1:8">
+      <c r="J10" s="10"/>
+    </row>
+    <row r="11" spans="1:10">
       <c r="A11" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="10">
+      <c r="D11" s="11">
         <v>0.08333333333333333</v>
       </c>
-      <c r="C11" s="10">
+      <c r="E11" s="11">
         <v>0.08333333333333333</v>
       </c>
-      <c r="D11" s="10">
+      <c r="F11" s="11">
         <v>0.08333333333333333</v>
       </c>
-      <c r="G11" s="11" t="s">
+      <c r="I11" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="H11" s="11"/>
-    </row>
-    <row r="12" spans="1:8">
+      <c r="J11" s="10"/>
+    </row>
+    <row r="12" spans="1:10">
       <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="B12" s="10">
+      <c r="D12" s="11">
         <v>0.1666666666666667</v>
       </c>
-      <c r="C12" s="10">
+      <c r="E12" s="11">
         <v>0.1666666666666667</v>
       </c>
-      <c r="D12" s="10">
+      <c r="F12" s="11">
         <v>0.1666666666666667</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:10">
       <c r="A13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="B13" s="10">
+      <c r="D13" s="11">
         <v>0.08333333333333333</v>
       </c>
-      <c r="C13" s="10">
+      <c r="E13" s="11">
         <v>0.08333333333333333</v>
       </c>
-      <c r="D13" s="10">
+      <c r="F13" s="11">
         <v>0.08333333333333333</v>
       </c>
-      <c r="G13" s="11" t="s">
+      <c r="I13" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="H13" s="11"/>
-    </row>
-    <row r="14" spans="1:8">
+      <c r="J13" s="10"/>
+    </row>
+    <row r="14" spans="1:10">
       <c r="A14" t="s">
+        <v>35</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="10">
+      <c r="D14" s="11">
         <v>0.08333333333333333</v>
       </c>
-      <c r="C14" s="10">
+      <c r="E14" s="11">
         <v>0.08333333333333333</v>
       </c>
-      <c r="D14" s="10">
+      <c r="F14" s="11">
         <v>0.08333333333333333</v>
       </c>
-      <c r="G14" s="11" t="s">
+      <c r="I14" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="H14" s="11"/>
-    </row>
-    <row r="15" spans="1:8">
+      <c r="J14" s="10"/>
+    </row>
+    <row r="15" spans="1:10">
       <c r="A15" t="s">
+        <v>35</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B15" s="10">
+      <c r="D15" s="11">
         <v>0.08333333333333333</v>
       </c>
-      <c r="C15" s="10">
+      <c r="E15" s="11">
         <v>0.08333333333333333</v>
       </c>
-      <c r="D15" s="10">
+      <c r="F15" s="11">
         <v>0.08333333333333333</v>
       </c>
-      <c r="G15" s="11" t="s">
+      <c r="I15" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="H15" s="11"/>
-    </row>
-    <row r="16" spans="1:8">
+      <c r="J15" s="10"/>
+    </row>
+    <row r="16" spans="1:10">
       <c r="A16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="B16" s="10">
+      <c r="D16" s="11">
         <v>0.08333333333333333</v>
       </c>
-      <c r="C16" s="10">
+      <c r="E16" s="11">
         <v>0.08333333333333333</v>
       </c>
-      <c r="D16" s="10">
+      <c r="F16" s="11">
         <v>0.08333333333333333</v>
       </c>
-      <c r="G16" s="11" t="s">
+      <c r="I16" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="H16" s="11"/>
+      <c r="J16" s="10"/>
     </row>
     <row r="19" spans="1:7">
       <c r="A19" s="12" t="s">
@@ -4922,7 +5006,7 @@
     <mergeCell ref="A24:G24"/>
     <mergeCell ref="A25:G25"/>
   </mergeCells>
-  <conditionalFormatting sqref="A3:H16">
+  <conditionalFormatting sqref="A3:J16">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>TRUE</formula>
     </cfRule>

</xml_diff>